<commit_message>
Stop tracking outputs y rds; usar .gitignore
</commit_message>
<xml_diff>
--- a/R/Analisis_NAs_4CCAA.xlsx
+++ b/R/Analisis_NAs_4CCAA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/841d1d890aeb2523/Documentos/MATEMÁTICAS URJC/CUARTO CURSO/TFG/tfg_composite_indicators/R/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_79FDE8D64D7B820CE23FDEE83C9F27AF405474C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5BDFE53-E283-415C-B596-2077832FDE71}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="11_79FDE8D64D0B0D468E5DC4E83C9F27AF405474C8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{001EAE1B-B626-4108-8505-C6CD4572628C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11280" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="58">
   <si>
     <t>indicator_id</t>
   </si>
@@ -197,6 +197,9 @@
   <si>
     <t>ISOC0013</t>
   </si>
+  <si>
+    <t>NO EXISTE</t>
+  </si>
 </sst>
 </file>
 
@@ -217,18 +220,12 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -243,10 +240,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -254,11 +250,11 @@
   <dxfs count="8">
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1565,10 +1561,18 @@
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="B2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E2" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -2438,8 +2442,13 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:E53">
-    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="1">
+  <conditionalFormatting sqref="B3:E53">
+    <cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="1">
+      <formula>NOT(ISERROR(SEARCH("1",B3)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:E2">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="1">
       <formula>NOT(ISERROR(SEARCH("1",B2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4308,10 +4317,18 @@
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="B2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E2" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -5181,8 +5198,13 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:E53">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="1">
+  <conditionalFormatting sqref="B3:E53">
+    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="1">
+      <formula>NOT(ISERROR(SEARCH("1",B3)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B2:E2">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="1">
       <formula>NOT(ISERROR(SEARCH("1",B2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5217,10 +5239,18 @@
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="B2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E2" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -6091,13 +6121,8 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:E53">
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="1">
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="1">
       <formula>NOT(ISERROR(SEARCH("1",B2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:E2">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text=" ">
-      <formula>NOT(ISERROR(SEARCH(" ",B2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>